<commit_message>
Visão geral: valores à esquerda nas tabelas e planilha de vendas atualizada
- Tabelas Estoque e Vendas com valores alinhados à esquerda
- Planilha de vendas atualizada

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modelo-painel-vendas.xlsx
+++ b/modelo-painel-vendas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filip\OneDrive\Área de Trabalho\SALES DASHBOARD - CLAUDE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{061EF26C-AF64-48E8-BA79-9F289E460106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1733FD8-240B-4F22-8F7D-716ED213EFAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
     <sheet name="Instruções" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Unidades!$A$1:$I$647</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Unidades!$A$1:$I$648</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Unidades!$C$1:$H$140</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="789" uniqueCount="182">
   <si>
     <t>Empreendimento</t>
   </si>
@@ -574,6 +574,15 @@
   </si>
   <si>
     <t>Marilene</t>
+  </si>
+  <si>
+    <t>Ricardo Aparecido da Silva</t>
+  </si>
+  <si>
+    <t>210 - BL 1</t>
+  </si>
+  <si>
+    <t>Plano 24x</t>
   </si>
 </sst>
 </file>
@@ -1004,8 +1013,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:J647"/>
+  <dimension ref="A1:J651"/>
   <sheetFormatPr defaultRowHeight="12" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5" style="1" bestFit="1" customWidth="1"/>
@@ -1053,7 +1061,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="2" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="9">
         <v>44958</v>
       </c>
@@ -1081,7 +1089,7 @@
       </c>
       <c r="J2" s="6"/>
     </row>
-    <row r="3" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="9">
         <v>44958</v>
       </c>
@@ -1109,7 +1117,7 @@
       </c>
       <c r="J3" s="6"/>
     </row>
-    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>45292</v>
       </c>
@@ -1137,7 +1145,7 @@
       </c>
       <c r="J4" s="6"/>
     </row>
-    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="9">
         <v>45352</v>
       </c>
@@ -1165,7 +1173,7 @@
       </c>
       <c r="J5" s="6"/>
     </row>
-    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="9">
         <v>44621</v>
       </c>
@@ -1193,7 +1201,7 @@
       </c>
       <c r="J6" s="6"/>
     </row>
-    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="9">
         <v>44958</v>
       </c>
@@ -1221,7 +1229,7 @@
       </c>
       <c r="J7" s="6"/>
     </row>
-    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="9">
         <v>44621</v>
       </c>
@@ -1249,7 +1257,7 @@
       </c>
       <c r="J8" s="6"/>
     </row>
-    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="9">
         <v>44652</v>
       </c>
@@ -1277,7 +1285,7 @@
       </c>
       <c r="J9" s="6"/>
     </row>
-    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="9">
         <v>44652</v>
       </c>
@@ -1305,7 +1313,7 @@
       </c>
       <c r="J10" s="6"/>
     </row>
-    <row r="11" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="9">
         <v>45292</v>
       </c>
@@ -1333,7 +1341,7 @@
       </c>
       <c r="J11" s="6"/>
     </row>
-    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="9">
         <v>44927</v>
       </c>
@@ -1361,7 +1369,7 @@
       </c>
       <c r="J12" s="6"/>
     </row>
-    <row r="13" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="9">
         <v>45292</v>
       </c>
@@ -1389,7 +1397,7 @@
       </c>
       <c r="J13" s="6"/>
     </row>
-    <row r="14" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="9">
         <v>45231</v>
       </c>
@@ -1417,7 +1425,7 @@
       </c>
       <c r="J14" s="6"/>
     </row>
-    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="9">
         <v>44866</v>
       </c>
@@ -1445,7 +1453,7 @@
       </c>
       <c r="J15" s="6"/>
     </row>
-    <row r="16" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="9">
         <v>44621</v>
       </c>
@@ -1473,7 +1481,7 @@
       </c>
       <c r="J16" s="6"/>
     </row>
-    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="9">
         <v>44621</v>
       </c>
@@ -1501,7 +1509,7 @@
       </c>
       <c r="J17" s="6"/>
     </row>
-    <row r="18" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
         <v>44927</v>
       </c>
@@ -1529,7 +1537,7 @@
       </c>
       <c r="J18" s="6"/>
     </row>
-    <row r="19" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="9">
         <v>44621</v>
       </c>
@@ -1557,7 +1565,7 @@
       </c>
       <c r="J19" s="6"/>
     </row>
-    <row r="20" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="9">
         <v>44621</v>
       </c>
@@ -1585,7 +1593,7 @@
       </c>
       <c r="J20" s="6"/>
     </row>
-    <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="9">
         <v>44682</v>
       </c>
@@ -1613,7 +1621,7 @@
       </c>
       <c r="J21" s="6"/>
     </row>
-    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="9">
         <v>44621</v>
       </c>
@@ -1641,7 +1649,7 @@
       </c>
       <c r="J22" s="6"/>
     </row>
-    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="9">
         <v>44774</v>
       </c>
@@ -1669,7 +1677,7 @@
       </c>
       <c r="J23" s="6"/>
     </row>
-    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="9">
         <v>44896</v>
       </c>
@@ -1697,7 +1705,7 @@
       </c>
       <c r="J24" s="6"/>
     </row>
-    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="9">
         <v>44927</v>
       </c>
@@ -1725,7 +1733,7 @@
       </c>
       <c r="J25" s="6"/>
     </row>
-    <row r="26" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="9">
         <v>44835</v>
       </c>
@@ -1753,7 +1761,7 @@
       </c>
       <c r="J26" s="6"/>
     </row>
-    <row r="27" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="9">
         <v>45139</v>
       </c>
@@ -1781,7 +1789,7 @@
       </c>
       <c r="J27" s="6"/>
     </row>
-    <row r="28" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="9">
         <v>44958</v>
       </c>
@@ -1809,7 +1817,7 @@
       </c>
       <c r="J28" s="6"/>
     </row>
-    <row r="29" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="9">
         <v>45352</v>
       </c>
@@ -1837,7 +1845,7 @@
       </c>
       <c r="J29" s="6"/>
     </row>
-    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="9">
         <v>45406</v>
       </c>
@@ -1865,7 +1873,7 @@
       </c>
       <c r="J30" s="6"/>
     </row>
-    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="9">
         <v>45352</v>
       </c>
@@ -1893,7 +1901,7 @@
       </c>
       <c r="J31" s="6"/>
     </row>
-    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="9">
         <v>45387</v>
       </c>
@@ -1921,7 +1929,7 @@
       </c>
       <c r="J32" s="6"/>
     </row>
-    <row r="33" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="9">
         <v>45323</v>
       </c>
@@ -1949,7 +1957,7 @@
       </c>
       <c r="J33" s="6"/>
     </row>
-    <row r="34" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="9">
         <v>45352</v>
       </c>
@@ -1975,7 +1983,7 @@
       </c>
       <c r="J34" s="6"/>
     </row>
-    <row r="35" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="9">
         <v>45386</v>
       </c>
@@ -2001,7 +2009,7 @@
       </c>
       <c r="J35" s="6"/>
     </row>
-    <row r="36" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="9">
         <v>45323</v>
       </c>
@@ -2027,7 +2035,7 @@
       </c>
       <c r="J36" s="6"/>
     </row>
-    <row r="37" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="9">
         <v>45352</v>
       </c>
@@ -2053,7 +2061,7 @@
       </c>
       <c r="J37" s="6"/>
     </row>
-    <row r="38" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="9">
         <v>45413</v>
       </c>
@@ -2081,7 +2089,7 @@
       </c>
       <c r="J38" s="6"/>
     </row>
-    <row r="39" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="9">
         <v>45413</v>
       </c>
@@ -2109,7 +2117,7 @@
       </c>
       <c r="J39" s="6"/>
     </row>
-    <row r="40" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="9">
         <v>45413</v>
       </c>
@@ -2137,7 +2145,7 @@
       </c>
       <c r="J40" s="6"/>
     </row>
-    <row r="41" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="9">
         <v>45474</v>
       </c>
@@ -2165,7 +2173,7 @@
       </c>
       <c r="J41" s="6"/>
     </row>
-    <row r="42" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="9">
         <v>45499</v>
       </c>
@@ -2191,7 +2199,7 @@
       </c>
       <c r="J42" s="6"/>
     </row>
-    <row r="43" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="9">
         <v>45534</v>
       </c>
@@ -2217,7 +2225,7 @@
       </c>
       <c r="J43" s="6"/>
     </row>
-    <row r="44" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="9">
         <v>45579</v>
       </c>
@@ -2245,7 +2253,7 @@
       </c>
       <c r="J44" s="6"/>
     </row>
-    <row r="45" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="9">
         <v>45573</v>
       </c>
@@ -2273,7 +2281,7 @@
       </c>
       <c r="J45" s="6"/>
     </row>
-    <row r="46" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="9">
         <v>45576</v>
       </c>
@@ -2301,7 +2309,7 @@
       </c>
       <c r="J46" s="6"/>
     </row>
-    <row r="47" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="9">
         <v>45566</v>
       </c>
@@ -2329,7 +2337,7 @@
       </c>
       <c r="J47" s="6"/>
     </row>
-    <row r="48" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="9">
         <v>45566</v>
       </c>
@@ -2357,7 +2365,7 @@
       </c>
       <c r="J48" s="6"/>
     </row>
-    <row r="49" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="9">
         <v>45581</v>
       </c>
@@ -2385,7 +2393,7 @@
       </c>
       <c r="J49" s="6"/>
     </row>
-    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="9">
         <v>45603</v>
       </c>
@@ -2413,7 +2421,7 @@
       </c>
       <c r="J50" s="6"/>
     </row>
-    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="9">
         <v>45644</v>
       </c>
@@ -2441,7 +2449,7 @@
       </c>
       <c r="J51" s="6"/>
     </row>
-    <row r="52" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="9">
         <v>45659</v>
       </c>
@@ -2469,7 +2477,7 @@
       </c>
       <c r="J52" s="6"/>
     </row>
-    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="9">
         <v>45659</v>
       </c>
@@ -2497,7 +2505,7 @@
       </c>
       <c r="J53" s="6"/>
     </row>
-    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="9">
         <v>45659</v>
       </c>
@@ -2523,7 +2531,7 @@
       </c>
       <c r="J54" s="6"/>
     </row>
-    <row r="55" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="9">
         <v>45679</v>
       </c>
@@ -2551,7 +2559,7 @@
       </c>
       <c r="J55" s="6"/>
     </row>
-    <row r="56" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="9">
         <v>45713</v>
       </c>
@@ -2579,7 +2587,7 @@
       </c>
       <c r="J56" s="6"/>
     </row>
-    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="9">
         <v>45726</v>
       </c>
@@ -2607,7 +2615,7 @@
       </c>
       <c r="J57" s="6"/>
     </row>
-    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="9">
         <v>45724</v>
       </c>
@@ -2635,7 +2643,7 @@
       </c>
       <c r="J58" s="6"/>
     </row>
-    <row r="59" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="9">
         <v>45726</v>
       </c>
@@ -2663,7 +2671,7 @@
       </c>
       <c r="J59" s="6"/>
     </row>
-    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="9">
         <v>45738</v>
       </c>
@@ -2691,7 +2699,7 @@
       </c>
       <c r="J60" s="6"/>
     </row>
-    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="9">
         <v>45783</v>
       </c>
@@ -2719,7 +2727,7 @@
       </c>
       <c r="J61" s="6"/>
     </row>
-    <row r="62" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="9">
         <v>45860</v>
       </c>
@@ -2745,7 +2753,7 @@
       </c>
       <c r="J62" s="6"/>
     </row>
-    <row r="63" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="9">
         <v>45888</v>
       </c>
@@ -2771,7 +2779,7 @@
       </c>
       <c r="J63" s="6"/>
     </row>
-    <row r="64" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="9">
         <v>45909</v>
       </c>
@@ -2799,7 +2807,7 @@
       </c>
       <c r="J64" s="6"/>
     </row>
-    <row r="65" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="9">
         <v>45909</v>
       </c>
@@ -2827,7 +2835,7 @@
       </c>
       <c r="J65" s="6"/>
     </row>
-    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="9">
         <v>45954</v>
       </c>
@@ -2853,7 +2861,7 @@
       </c>
       <c r="J66" s="6"/>
     </row>
-    <row r="67" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" s="9">
         <v>45966</v>
       </c>
@@ -2881,7 +2889,7 @@
       </c>
       <c r="J67" s="6"/>
     </row>
-    <row r="68" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="9">
         <v>46028</v>
       </c>
@@ -2907,7 +2915,7 @@
       </c>
       <c r="J68" s="6"/>
     </row>
-    <row r="69" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="9">
         <v>46031</v>
       </c>
@@ -2933,7 +2941,7 @@
       </c>
       <c r="J69" s="6"/>
     </row>
-    <row r="70" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" s="9">
         <v>46034</v>
       </c>
@@ -2961,7 +2969,7 @@
       </c>
       <c r="J70" s="6"/>
     </row>
-    <row r="71" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" s="9">
         <v>46036</v>
       </c>
@@ -2989,7 +2997,7 @@
       </c>
       <c r="J71" s="6"/>
     </row>
-    <row r="72" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" s="9">
         <v>46038</v>
       </c>
@@ -3015,7 +3023,7 @@
       </c>
       <c r="J72" s="6"/>
     </row>
-    <row r="73" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" s="9">
         <v>46032</v>
       </c>
@@ -3043,7 +3051,7 @@
       </c>
       <c r="J73" s="6"/>
     </row>
-    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" s="9">
         <v>46043</v>
       </c>
@@ -3071,7 +3079,7 @@
       </c>
       <c r="J74" s="6"/>
     </row>
-    <row r="75" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" s="9">
         <v>46060</v>
       </c>
@@ -3099,7 +3107,7 @@
       </c>
       <c r="J75" s="6"/>
     </row>
-    <row r="76" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" s="9">
         <v>46045</v>
       </c>
@@ -3127,7 +3135,7 @@
       </c>
       <c r="J76" s="6"/>
     </row>
-    <row r="77" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" s="9">
         <v>46058</v>
       </c>
@@ -3153,7 +3161,7 @@
       </c>
       <c r="J77" s="6"/>
     </row>
-    <row r="78" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" s="9">
         <v>46083</v>
       </c>
@@ -3181,7 +3189,7 @@
       </c>
       <c r="J78" s="6"/>
     </row>
-    <row r="79" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" s="9">
         <v>46107</v>
       </c>
@@ -3207,7 +3215,7 @@
       </c>
       <c r="J79" s="6"/>
     </row>
-    <row r="80" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" s="9">
         <v>46120</v>
       </c>
@@ -3235,7 +3243,7 @@
       </c>
       <c r="J80" s="6"/>
     </row>
-    <row r="81" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" s="9">
         <v>46090</v>
       </c>
@@ -3263,7 +3271,7 @@
       </c>
       <c r="J81" s="6"/>
     </row>
-    <row r="82" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" s="9">
         <v>46185</v>
       </c>
@@ -3289,7 +3297,7 @@
       </c>
       <c r="J82" s="6"/>
     </row>
-    <row r="83" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" s="9">
         <v>46209</v>
       </c>
@@ -3317,7 +3325,7 @@
       </c>
       <c r="J83" s="6"/>
     </row>
-    <row r="84" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" s="9">
         <v>46183</v>
       </c>
@@ -3345,7 +3353,7 @@
       </c>
       <c r="J84" s="6"/>
     </row>
-    <row r="85" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" s="9">
         <v>46261</v>
       </c>
@@ -3373,7 +3381,7 @@
       </c>
       <c r="J85" s="6"/>
     </row>
-    <row r="86" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A86" s="9">
         <v>46275</v>
       </c>
@@ -5038,2038 +5046,2074 @@
         <v>99</v>
       </c>
     </row>
-    <row r="142" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A142" s="7"/>
-      <c r="H142" s="3"/>
-    </row>
-    <row r="143" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A142" s="7">
+        <v>46318</v>
+      </c>
+      <c r="B142" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C142" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="D142" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="E142" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F142" s="1">
+        <v>74.61</v>
+      </c>
+      <c r="G142" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H142" s="3">
+        <v>621738.23999999999</v>
+      </c>
+      <c r="I142" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="J142" s="1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A143" s="7"/>
       <c r="H143" s="3"/>
     </row>
-    <row r="144" spans="1:10" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A144" s="7"/>
       <c r="H144" s="3"/>
     </row>
-    <row r="145" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A145" s="7"/>
       <c r="H145" s="3"/>
     </row>
-    <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A146" s="7"/>
       <c r="H146" s="3"/>
     </row>
-    <row r="147" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A147" s="7"/>
       <c r="H147" s="3"/>
     </row>
-    <row r="148" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A148" s="7"/>
       <c r="H148" s="3"/>
     </row>
-    <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A149" s="7"/>
       <c r="H149" s="3"/>
     </row>
-    <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A150" s="7"/>
       <c r="H150" s="3"/>
     </row>
-    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A151" s="7"/>
       <c r="H151" s="3"/>
     </row>
-    <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A152" s="7"/>
       <c r="H152" s="3"/>
     </row>
-    <row r="153" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A153" s="7"/>
       <c r="H153" s="3"/>
     </row>
-    <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A154" s="7"/>
       <c r="H154" s="3"/>
     </row>
-    <row r="155" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A155" s="7"/>
       <c r="H155" s="3"/>
     </row>
-    <row r="156" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A156" s="7"/>
       <c r="H156" s="3"/>
     </row>
-    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A157" s="7"/>
       <c r="H157" s="3"/>
     </row>
-    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A158" s="7"/>
       <c r="H158" s="3"/>
     </row>
-    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A159" s="7"/>
       <c r="H159" s="3"/>
     </row>
-    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A160" s="7"/>
       <c r="H160" s="3"/>
     </row>
-    <row r="161" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A161" s="7"/>
       <c r="H161" s="3"/>
     </row>
-    <row r="162" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A162" s="7"/>
       <c r="H162" s="3"/>
     </row>
-    <row r="163" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A163" s="7"/>
       <c r="H163" s="3"/>
     </row>
-    <row r="164" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A164" s="7"/>
       <c r="H164" s="3"/>
     </row>
-    <row r="165" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A165" s="7"/>
       <c r="H165" s="3"/>
     </row>
-    <row r="166" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A166" s="7"/>
       <c r="H166" s="3"/>
     </row>
-    <row r="167" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A167" s="7"/>
       <c r="H167" s="3"/>
     </row>
-    <row r="168" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A168" s="7"/>
       <c r="H168" s="3"/>
     </row>
-    <row r="169" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A169" s="7"/>
       <c r="H169" s="3"/>
     </row>
-    <row r="170" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A170" s="7"/>
       <c r="H170" s="3"/>
     </row>
-    <row r="171" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A171" s="7"/>
       <c r="H171" s="3"/>
     </row>
-    <row r="172" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A172" s="7"/>
       <c r="H172" s="3"/>
     </row>
-    <row r="173" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A173" s="7"/>
       <c r="H173" s="3"/>
     </row>
-    <row r="174" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A174" s="7"/>
       <c r="H174" s="3"/>
     </row>
-    <row r="175" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A175" s="7"/>
       <c r="H175" s="3"/>
     </row>
-    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A176" s="7"/>
       <c r="H176" s="3"/>
     </row>
-    <row r="177" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A177" s="7"/>
       <c r="H177" s="3"/>
     </row>
-    <row r="178" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A178" s="7"/>
       <c r="H178" s="3"/>
     </row>
-    <row r="179" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A179" s="7"/>
       <c r="H179" s="3"/>
     </row>
-    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A180" s="7"/>
       <c r="H180" s="3"/>
     </row>
-    <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A181" s="7"/>
       <c r="H181" s="3"/>
     </row>
-    <row r="182" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A182" s="7"/>
       <c r="H182" s="3"/>
     </row>
-    <row r="183" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A183" s="7"/>
       <c r="H183" s="3"/>
     </row>
-    <row r="184" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A184" s="7"/>
       <c r="H184" s="3"/>
     </row>
-    <row r="185" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A185" s="7"/>
       <c r="H185" s="3"/>
     </row>
-    <row r="186" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A186" s="7"/>
       <c r="H186" s="3"/>
     </row>
-    <row r="187" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A187" s="7"/>
       <c r="H187" s="3"/>
     </row>
-    <row r="188" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A188" s="7"/>
       <c r="H188" s="3"/>
     </row>
-    <row r="189" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A189" s="7"/>
       <c r="H189" s="3"/>
     </row>
-    <row r="190" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A190" s="7"/>
       <c r="H190" s="3"/>
     </row>
-    <row r="191" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A191" s="7"/>
       <c r="H191" s="3"/>
     </row>
-    <row r="192" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A192" s="7"/>
       <c r="H192" s="3"/>
     </row>
-    <row r="193" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A193" s="7"/>
       <c r="H193" s="3"/>
     </row>
-    <row r="194" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A194" s="7"/>
       <c r="H194" s="3"/>
     </row>
-    <row r="195" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A195" s="7"/>
       <c r="H195" s="3"/>
     </row>
-    <row r="196" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A196" s="7"/>
       <c r="H196" s="3"/>
     </row>
-    <row r="197" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A197" s="7"/>
       <c r="H197" s="3"/>
     </row>
-    <row r="198" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A198" s="7"/>
       <c r="H198" s="3"/>
     </row>
-    <row r="199" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A199" s="7"/>
       <c r="H199" s="3"/>
     </row>
-    <row r="200" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A200" s="7"/>
       <c r="H200" s="3"/>
     </row>
-    <row r="201" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A201" s="7"/>
       <c r="H201" s="3"/>
     </row>
-    <row r="202" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A202" s="7"/>
       <c r="H202" s="3"/>
     </row>
-    <row r="203" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A203" s="7"/>
       <c r="H203" s="3"/>
     </row>
-    <row r="204" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A204" s="7"/>
       <c r="H204" s="3"/>
     </row>
-    <row r="205" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A205" s="7"/>
       <c r="H205" s="3"/>
     </row>
-    <row r="206" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A206" s="7"/>
       <c r="H206" s="3"/>
     </row>
-    <row r="207" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A207" s="7"/>
       <c r="H207" s="3"/>
     </row>
-    <row r="208" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A208" s="7"/>
       <c r="H208" s="3"/>
     </row>
-    <row r="209" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A209" s="7"/>
       <c r="H209" s="3"/>
     </row>
-    <row r="210" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A210" s="7"/>
       <c r="H210" s="3"/>
     </row>
-    <row r="211" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A211" s="7"/>
       <c r="H211" s="3"/>
     </row>
-    <row r="212" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A212" s="7"/>
       <c r="H212" s="3"/>
     </row>
-    <row r="213" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A213" s="7"/>
       <c r="H213" s="3"/>
     </row>
-    <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A214" s="7"/>
       <c r="H214" s="3"/>
     </row>
-    <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A215" s="7"/>
       <c r="H215" s="3"/>
     </row>
-    <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A216" s="7"/>
       <c r="H216" s="3"/>
     </row>
-    <row r="217" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A217" s="7"/>
       <c r="H217" s="3"/>
     </row>
-    <row r="218" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A218" s="7"/>
       <c r="H218" s="3"/>
     </row>
-    <row r="219" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A219" s="7"/>
       <c r="H219" s="3"/>
     </row>
-    <row r="220" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A220" s="7"/>
       <c r="H220" s="3"/>
     </row>
-    <row r="221" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A221" s="7"/>
       <c r="H221" s="3"/>
     </row>
-    <row r="222" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A222" s="7"/>
       <c r="H222" s="3"/>
     </row>
-    <row r="223" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A223" s="7"/>
       <c r="H223" s="3"/>
     </row>
-    <row r="224" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A224" s="7"/>
       <c r="H224" s="3"/>
     </row>
-    <row r="225" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A225" s="7"/>
       <c r="H225" s="3"/>
     </row>
-    <row r="226" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A226" s="7"/>
       <c r="H226" s="3"/>
     </row>
-    <row r="227" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A227" s="7"/>
       <c r="H227" s="3"/>
     </row>
-    <row r="228" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A228" s="7"/>
       <c r="H228" s="3"/>
     </row>
-    <row r="229" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A229" s="7"/>
       <c r="H229" s="3"/>
     </row>
-    <row r="230" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A230" s="7"/>
       <c r="H230" s="3"/>
     </row>
-    <row r="231" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A231" s="7"/>
       <c r="H231" s="3"/>
     </row>
-    <row r="232" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A232" s="7"/>
       <c r="H232" s="3"/>
     </row>
-    <row r="233" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A233" s="7"/>
       <c r="H233" s="3"/>
     </row>
-    <row r="234" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A234" s="7"/>
       <c r="H234" s="3"/>
     </row>
-    <row r="235" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A235" s="7"/>
       <c r="H235" s="3"/>
     </row>
-    <row r="236" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A236" s="7"/>
       <c r="H236" s="3"/>
     </row>
-    <row r="237" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A237" s="7"/>
       <c r="H237" s="3"/>
     </row>
-    <row r="238" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A238" s="7"/>
       <c r="H238" s="3"/>
     </row>
-    <row r="239" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A239" s="7"/>
       <c r="H239" s="3"/>
     </row>
-    <row r="240" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A240" s="7"/>
       <c r="H240" s="3"/>
     </row>
-    <row r="241" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A241" s="7"/>
       <c r="H241" s="3"/>
     </row>
-    <row r="242" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A242" s="7"/>
       <c r="H242" s="3"/>
     </row>
-    <row r="243" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A243" s="7"/>
       <c r="H243" s="3"/>
     </row>
-    <row r="244" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A244" s="7"/>
       <c r="H244" s="3"/>
     </row>
-    <row r="245" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A245" s="7"/>
       <c r="H245" s="3"/>
     </row>
-    <row r="246" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A246" s="7"/>
       <c r="H246" s="3"/>
     </row>
-    <row r="247" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A247" s="7"/>
       <c r="H247" s="3"/>
     </row>
-    <row r="248" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A248" s="7"/>
       <c r="H248" s="3"/>
     </row>
-    <row r="249" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A249" s="7"/>
       <c r="H249" s="3"/>
     </row>
-    <row r="250" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A250" s="7"/>
       <c r="H250" s="3"/>
     </row>
-    <row r="251" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A251" s="7"/>
       <c r="H251" s="3"/>
     </row>
-    <row r="252" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A252" s="7"/>
       <c r="H252" s="3"/>
     </row>
-    <row r="253" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A253" s="7"/>
       <c r="H253" s="3"/>
     </row>
-    <row r="254" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A254" s="7"/>
       <c r="H254" s="3"/>
     </row>
-    <row r="255" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A255" s="7"/>
       <c r="H255" s="3"/>
     </row>
-    <row r="256" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A256" s="7"/>
       <c r="H256" s="3"/>
     </row>
-    <row r="257" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A257" s="7"/>
       <c r="H257" s="3"/>
     </row>
-    <row r="258" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A258" s="7"/>
       <c r="H258" s="3"/>
     </row>
-    <row r="259" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A259" s="7"/>
       <c r="H259" s="3"/>
     </row>
-    <row r="260" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A260" s="7"/>
       <c r="H260" s="3"/>
     </row>
-    <row r="261" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A261" s="7"/>
       <c r="H261" s="3"/>
     </row>
-    <row r="262" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A262" s="7"/>
       <c r="H262" s="3"/>
     </row>
-    <row r="263" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A263" s="7"/>
       <c r="H263" s="3"/>
     </row>
-    <row r="264" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A264" s="7"/>
       <c r="H264" s="3"/>
     </row>
-    <row r="265" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A265" s="7"/>
       <c r="H265" s="3"/>
     </row>
-    <row r="266" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A266" s="7"/>
       <c r="H266" s="3"/>
     </row>
-    <row r="267" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A267" s="7"/>
       <c r="H267" s="3"/>
     </row>
-    <row r="268" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A268" s="7"/>
       <c r="H268" s="3"/>
     </row>
-    <row r="269" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A269" s="7"/>
       <c r="H269" s="3"/>
     </row>
-    <row r="270" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A270" s="7"/>
       <c r="H270" s="3"/>
     </row>
-    <row r="271" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A271" s="7"/>
       <c r="H271" s="3"/>
     </row>
-    <row r="272" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A272" s="7"/>
       <c r="H272" s="3"/>
     </row>
-    <row r="273" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A273" s="7"/>
       <c r="H273" s="3"/>
     </row>
-    <row r="274" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A274" s="7"/>
       <c r="H274" s="3"/>
     </row>
-    <row r="275" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A275" s="7"/>
       <c r="H275" s="3"/>
     </row>
-    <row r="276" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A276" s="7"/>
       <c r="H276" s="3"/>
     </row>
-    <row r="277" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A277" s="7"/>
       <c r="H277" s="3"/>
     </row>
-    <row r="278" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A278" s="7"/>
       <c r="H278" s="3"/>
     </row>
-    <row r="279" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A279" s="7"/>
       <c r="H279" s="3"/>
     </row>
-    <row r="280" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A280" s="7"/>
       <c r="H280" s="3"/>
     </row>
-    <row r="281" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A281" s="7"/>
       <c r="H281" s="3"/>
     </row>
-    <row r="282" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A282" s="7"/>
       <c r="H282" s="3"/>
     </row>
-    <row r="283" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A283" s="7"/>
       <c r="H283" s="3"/>
     </row>
-    <row r="284" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A284" s="7"/>
       <c r="H284" s="3"/>
     </row>
-    <row r="285" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A285" s="7"/>
       <c r="H285" s="3"/>
     </row>
-    <row r="286" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A286" s="7"/>
       <c r="H286" s="3"/>
     </row>
-    <row r="287" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A287" s="7"/>
       <c r="H287" s="3"/>
     </row>
-    <row r="288" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A288" s="7"/>
       <c r="H288" s="3"/>
     </row>
-    <row r="289" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A289" s="7"/>
       <c r="H289" s="3"/>
     </row>
-    <row r="290" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A290" s="7"/>
       <c r="H290" s="3"/>
     </row>
-    <row r="291" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A291" s="7"/>
       <c r="H291" s="3"/>
     </row>
-    <row r="292" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A292" s="7"/>
       <c r="H292" s="3"/>
     </row>
-    <row r="293" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A293" s="7"/>
       <c r="H293" s="3"/>
     </row>
-    <row r="294" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A294" s="7"/>
       <c r="H294" s="3"/>
     </row>
-    <row r="295" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A295" s="7"/>
       <c r="H295" s="3"/>
     </row>
-    <row r="296" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A296" s="7"/>
       <c r="H296" s="3"/>
     </row>
-    <row r="297" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A297" s="7"/>
       <c r="H297" s="3"/>
     </row>
-    <row r="298" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A298" s="7"/>
       <c r="H298" s="3"/>
     </row>
-    <row r="299" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A299" s="7"/>
       <c r="H299" s="3"/>
     </row>
-    <row r="300" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A300" s="7"/>
       <c r="H300" s="3"/>
     </row>
-    <row r="301" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A301" s="7"/>
       <c r="H301" s="3"/>
     </row>
-    <row r="302" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A302" s="7"/>
       <c r="H302" s="3"/>
     </row>
-    <row r="303" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A303" s="7"/>
       <c r="H303" s="3"/>
     </row>
-    <row r="304" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A304" s="7"/>
       <c r="H304" s="3"/>
     </row>
-    <row r="305" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A305" s="7"/>
       <c r="H305" s="3"/>
     </row>
-    <row r="306" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A306" s="7"/>
       <c r="H306" s="3"/>
     </row>
-    <row r="307" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A307" s="7"/>
       <c r="H307" s="3"/>
     </row>
-    <row r="308" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A308" s="7"/>
       <c r="H308" s="3"/>
     </row>
-    <row r="309" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A309" s="7"/>
       <c r="H309" s="3"/>
     </row>
-    <row r="310" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A310" s="7"/>
       <c r="H310" s="3"/>
     </row>
-    <row r="311" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A311" s="7"/>
       <c r="H311" s="3"/>
     </row>
-    <row r="312" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A312" s="7"/>
       <c r="H312" s="3"/>
     </row>
-    <row r="313" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A313" s="7"/>
       <c r="H313" s="3"/>
     </row>
-    <row r="314" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A314" s="7"/>
       <c r="H314" s="3"/>
     </row>
-    <row r="315" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A315" s="7"/>
       <c r="H315" s="3"/>
     </row>
-    <row r="316" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A316" s="7"/>
       <c r="H316" s="3"/>
     </row>
-    <row r="317" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A317" s="7"/>
       <c r="H317" s="3"/>
     </row>
-    <row r="318" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A318" s="7"/>
       <c r="H318" s="3"/>
     </row>
-    <row r="319" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A319" s="7"/>
       <c r="H319" s="3"/>
     </row>
-    <row r="320" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A320" s="7"/>
       <c r="H320" s="3"/>
     </row>
-    <row r="321" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A321" s="7"/>
       <c r="H321" s="3"/>
     </row>
-    <row r="322" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A322" s="7"/>
       <c r="H322" s="3"/>
     </row>
-    <row r="323" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A323" s="7"/>
       <c r="H323" s="3"/>
     </row>
-    <row r="324" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A324" s="7"/>
       <c r="H324" s="3"/>
     </row>
-    <row r="325" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A325" s="7"/>
       <c r="H325" s="3"/>
     </row>
-    <row r="326" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A326" s="7"/>
       <c r="H326" s="3"/>
     </row>
-    <row r="327" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A327" s="7"/>
       <c r="H327" s="3"/>
     </row>
-    <row r="328" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A328" s="7"/>
       <c r="H328" s="3"/>
     </row>
-    <row r="329" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A329" s="7"/>
       <c r="H329" s="3"/>
     </row>
-    <row r="330" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A330" s="7"/>
       <c r="H330" s="3"/>
     </row>
-    <row r="331" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A331" s="7"/>
       <c r="H331" s="3"/>
     </row>
-    <row r="332" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A332" s="7"/>
       <c r="H332" s="3"/>
     </row>
-    <row r="333" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A333" s="7"/>
       <c r="H333" s="3"/>
     </row>
-    <row r="334" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A334" s="7"/>
       <c r="H334" s="3"/>
     </row>
-    <row r="335" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A335" s="7"/>
       <c r="H335" s="3"/>
     </row>
-    <row r="336" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A336" s="7"/>
       <c r="H336" s="3"/>
     </row>
-    <row r="337" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A337" s="7"/>
       <c r="H337" s="3"/>
     </row>
-    <row r="338" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A338" s="7"/>
       <c r="H338" s="3"/>
     </row>
-    <row r="339" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A339" s="7"/>
       <c r="H339" s="3"/>
     </row>
-    <row r="340" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A340" s="7"/>
       <c r="H340" s="3"/>
     </row>
-    <row r="341" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A341" s="7"/>
       <c r="H341" s="3"/>
     </row>
-    <row r="342" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A342" s="7"/>
       <c r="H342" s="3"/>
     </row>
-    <row r="343" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A343" s="7"/>
       <c r="H343" s="3"/>
     </row>
-    <row r="344" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A344" s="7"/>
       <c r="H344" s="3"/>
     </row>
-    <row r="345" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A345" s="7"/>
       <c r="H345" s="3"/>
     </row>
-    <row r="346" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A346" s="7"/>
       <c r="H346" s="3"/>
     </row>
-    <row r="347" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A347" s="7"/>
       <c r="H347" s="3"/>
     </row>
-    <row r="348" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A348" s="7"/>
       <c r="H348" s="3"/>
     </row>
-    <row r="349" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A349" s="7"/>
       <c r="H349" s="3"/>
     </row>
-    <row r="350" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A350" s="7"/>
       <c r="H350" s="3"/>
     </row>
-    <row r="351" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A351" s="7"/>
       <c r="H351" s="3"/>
     </row>
-    <row r="352" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A352" s="7"/>
       <c r="H352" s="3"/>
     </row>
-    <row r="353" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A353" s="7"/>
       <c r="H353" s="3"/>
     </row>
-    <row r="354" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A354" s="7"/>
       <c r="H354" s="3"/>
     </row>
-    <row r="355" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A355" s="7"/>
       <c r="H355" s="3"/>
     </row>
-    <row r="356" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A356" s="7"/>
       <c r="H356" s="3"/>
     </row>
-    <row r="357" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A357" s="7"/>
       <c r="H357" s="3"/>
     </row>
-    <row r="358" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A358" s="7"/>
       <c r="H358" s="3"/>
     </row>
-    <row r="359" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A359" s="7"/>
       <c r="H359" s="3"/>
     </row>
-    <row r="360" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A360" s="7"/>
       <c r="H360" s="3"/>
     </row>
-    <row r="361" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A361" s="7"/>
       <c r="H361" s="3"/>
     </row>
-    <row r="362" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A362" s="7"/>
       <c r="H362" s="3"/>
     </row>
-    <row r="363" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A363" s="7"/>
       <c r="H363" s="3"/>
     </row>
-    <row r="364" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A364" s="7"/>
       <c r="H364" s="3"/>
     </row>
-    <row r="365" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A365" s="7"/>
       <c r="H365" s="3"/>
     </row>
-    <row r="366" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A366" s="7"/>
       <c r="H366" s="3"/>
     </row>
-    <row r="367" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A367" s="7"/>
       <c r="H367" s="3"/>
     </row>
-    <row r="368" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A368" s="7"/>
       <c r="H368" s="3"/>
     </row>
-    <row r="369" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A369" s="7"/>
       <c r="H369" s="3"/>
     </row>
-    <row r="370" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A370" s="7"/>
       <c r="H370" s="3"/>
     </row>
-    <row r="371" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A371" s="7"/>
       <c r="H371" s="3"/>
     </row>
-    <row r="372" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A372" s="7"/>
       <c r="H372" s="3"/>
     </row>
-    <row r="373" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A373" s="7"/>
       <c r="H373" s="3"/>
     </row>
-    <row r="374" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A374" s="7"/>
       <c r="H374" s="3"/>
     </row>
-    <row r="375" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A375" s="7"/>
       <c r="H375" s="3"/>
     </row>
-    <row r="376" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A376" s="7"/>
       <c r="H376" s="3"/>
     </row>
-    <row r="377" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A377" s="7"/>
       <c r="H377" s="3"/>
     </row>
-    <row r="378" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A378" s="7"/>
       <c r="H378" s="3"/>
     </row>
-    <row r="379" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A379" s="7"/>
       <c r="H379" s="3"/>
     </row>
-    <row r="380" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A380" s="7"/>
       <c r="H380" s="3"/>
     </row>
-    <row r="381" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A381" s="7"/>
       <c r="H381" s="3"/>
     </row>
-    <row r="382" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A382" s="7"/>
       <c r="H382" s="3"/>
     </row>
-    <row r="383" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A383" s="7"/>
       <c r="H383" s="3"/>
     </row>
-    <row r="384" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A384" s="7"/>
       <c r="H384" s="3"/>
     </row>
-    <row r="385" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A385" s="7"/>
       <c r="H385" s="3"/>
     </row>
-    <row r="386" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A386" s="7"/>
       <c r="H386" s="3"/>
     </row>
-    <row r="387" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A387" s="7"/>
       <c r="H387" s="3"/>
     </row>
-    <row r="388" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A388" s="7"/>
       <c r="H388" s="3"/>
     </row>
-    <row r="389" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A389" s="7"/>
       <c r="H389" s="3"/>
     </row>
-    <row r="390" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A390" s="7"/>
       <c r="H390" s="3"/>
     </row>
-    <row r="391" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A391" s="7"/>
       <c r="H391" s="3"/>
     </row>
-    <row r="392" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A392" s="7"/>
       <c r="H392" s="3"/>
     </row>
-    <row r="393" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A393" s="7"/>
       <c r="H393" s="3"/>
     </row>
-    <row r="394" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A394" s="7"/>
       <c r="H394" s="3"/>
     </row>
-    <row r="395" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A395" s="7"/>
       <c r="H395" s="3"/>
     </row>
-    <row r="396" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A396" s="7"/>
       <c r="H396" s="3"/>
     </row>
-    <row r="397" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A397" s="7"/>
       <c r="H397" s="3"/>
     </row>
-    <row r="398" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A398" s="7"/>
       <c r="H398" s="3"/>
     </row>
-    <row r="399" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A399" s="7"/>
       <c r="H399" s="3"/>
     </row>
-    <row r="400" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A400" s="7"/>
       <c r="H400" s="3"/>
     </row>
-    <row r="401" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A401" s="7"/>
       <c r="H401" s="3"/>
     </row>
-    <row r="402" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A402" s="7"/>
       <c r="H402" s="3"/>
     </row>
-    <row r="403" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A403" s="7"/>
       <c r="H403" s="3"/>
     </row>
-    <row r="404" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A404" s="7"/>
       <c r="H404" s="3"/>
     </row>
-    <row r="405" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A405" s="7"/>
       <c r="H405" s="3"/>
     </row>
-    <row r="406" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A406" s="7"/>
       <c r="H406" s="3"/>
     </row>
-    <row r="407" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A407" s="7"/>
       <c r="H407" s="3"/>
     </row>
-    <row r="408" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A408" s="7"/>
       <c r="H408" s="3"/>
     </row>
-    <row r="409" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A409" s="7"/>
       <c r="H409" s="3"/>
     </row>
-    <row r="410" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A410" s="7"/>
       <c r="H410" s="3"/>
     </row>
-    <row r="411" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A411" s="7"/>
       <c r="H411" s="3"/>
     </row>
-    <row r="412" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A412" s="7"/>
       <c r="H412" s="3"/>
     </row>
-    <row r="413" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A413" s="7"/>
       <c r="H413" s="3"/>
     </row>
-    <row r="414" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A414" s="7"/>
       <c r="H414" s="3"/>
     </row>
-    <row r="415" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A415" s="7"/>
       <c r="H415" s="3"/>
     </row>
-    <row r="416" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A416" s="7"/>
       <c r="H416" s="3"/>
     </row>
-    <row r="417" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A417" s="7"/>
       <c r="H417" s="3"/>
     </row>
-    <row r="418" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A418" s="7"/>
       <c r="H418" s="3"/>
     </row>
-    <row r="419" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A419" s="7"/>
       <c r="H419" s="3"/>
     </row>
-    <row r="420" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A420" s="7"/>
       <c r="H420" s="3"/>
     </row>
-    <row r="421" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A421" s="7"/>
       <c r="H421" s="3"/>
     </row>
-    <row r="422" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A422" s="7"/>
       <c r="H422" s="3"/>
     </row>
-    <row r="423" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A423" s="7"/>
       <c r="H423" s="3"/>
     </row>
-    <row r="424" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A424" s="7"/>
       <c r="H424" s="3"/>
     </row>
-    <row r="425" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A425" s="7"/>
       <c r="H425" s="3"/>
     </row>
-    <row r="426" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A426" s="7"/>
       <c r="H426" s="3"/>
     </row>
-    <row r="427" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A427" s="7"/>
       <c r="H427" s="3"/>
     </row>
-    <row r="428" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A428" s="7"/>
       <c r="H428" s="3"/>
     </row>
-    <row r="429" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A429" s="7"/>
       <c r="H429" s="3"/>
     </row>
-    <row r="430" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A430" s="7"/>
       <c r="H430" s="3"/>
     </row>
-    <row r="431" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="431" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A431" s="7"/>
       <c r="H431" s="3"/>
     </row>
-    <row r="432" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A432" s="7"/>
       <c r="H432" s="3"/>
     </row>
-    <row r="433" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A433" s="7"/>
       <c r="H433" s="3"/>
     </row>
-    <row r="434" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A434" s="7"/>
       <c r="H434" s="3"/>
     </row>
-    <row r="435" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A435" s="7"/>
       <c r="H435" s="3"/>
     </row>
-    <row r="436" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A436" s="7"/>
       <c r="H436" s="3"/>
     </row>
-    <row r="437" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A437" s="7"/>
       <c r="H437" s="3"/>
     </row>
-    <row r="438" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A438" s="7"/>
       <c r="H438" s="3"/>
     </row>
-    <row r="439" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A439" s="7"/>
       <c r="H439" s="3"/>
     </row>
-    <row r="440" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A440" s="7"/>
       <c r="H440" s="3"/>
     </row>
-    <row r="441" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A441" s="7"/>
       <c r="H441" s="3"/>
     </row>
-    <row r="442" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A442" s="7"/>
       <c r="H442" s="3"/>
     </row>
-    <row r="443" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A443" s="7"/>
       <c r="H443" s="3"/>
     </row>
-    <row r="444" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="444" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A444" s="7"/>
       <c r="H444" s="3"/>
     </row>
-    <row r="445" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="445" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A445" s="7"/>
       <c r="H445" s="3"/>
     </row>
-    <row r="446" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A446" s="7"/>
       <c r="H446" s="3"/>
     </row>
-    <row r="447" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="447" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A447" s="7"/>
       <c r="H447" s="3"/>
     </row>
-    <row r="448" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="448" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A448" s="7"/>
       <c r="H448" s="3"/>
     </row>
-    <row r="449" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A449" s="7"/>
       <c r="H449" s="3"/>
     </row>
-    <row r="450" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A450" s="7"/>
       <c r="H450" s="3"/>
     </row>
-    <row r="451" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A451" s="7"/>
       <c r="H451" s="3"/>
     </row>
-    <row r="452" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A452" s="7"/>
       <c r="H452" s="3"/>
     </row>
-    <row r="453" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A453" s="7"/>
       <c r="H453" s="3"/>
     </row>
-    <row r="454" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="454" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A454" s="7"/>
       <c r="H454" s="3"/>
     </row>
-    <row r="455" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A455" s="7"/>
       <c r="H455" s="3"/>
     </row>
-    <row r="456" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A456" s="7"/>
       <c r="H456" s="3"/>
     </row>
-    <row r="457" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="457" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A457" s="7"/>
       <c r="H457" s="3"/>
     </row>
-    <row r="458" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A458" s="7"/>
       <c r="H458" s="3"/>
     </row>
-    <row r="459" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="459" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A459" s="7"/>
       <c r="H459" s="3"/>
     </row>
-    <row r="460" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="460" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A460" s="7"/>
       <c r="H460" s="3"/>
     </row>
-    <row r="461" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="461" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A461" s="7"/>
       <c r="H461" s="3"/>
     </row>
-    <row r="462" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A462" s="7"/>
       <c r="H462" s="3"/>
     </row>
-    <row r="463" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A463" s="7"/>
       <c r="H463" s="3"/>
     </row>
-    <row r="464" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A464" s="7"/>
       <c r="H464" s="3"/>
     </row>
-    <row r="465" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="465" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A465" s="7"/>
       <c r="H465" s="3"/>
     </row>
-    <row r="466" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="466" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A466" s="7"/>
       <c r="H466" s="3"/>
     </row>
-    <row r="467" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="467" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A467" s="7"/>
       <c r="H467" s="3"/>
     </row>
-    <row r="468" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="468" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A468" s="7"/>
       <c r="H468" s="3"/>
     </row>
-    <row r="469" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="469" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A469" s="7"/>
       <c r="H469" s="3"/>
     </row>
-    <row r="470" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A470" s="7"/>
       <c r="H470" s="3"/>
     </row>
-    <row r="471" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="471" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A471" s="7"/>
       <c r="H471" s="3"/>
     </row>
-    <row r="472" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="472" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A472" s="7"/>
       <c r="H472" s="3"/>
     </row>
-    <row r="473" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A473" s="7"/>
       <c r="H473" s="3"/>
     </row>
-    <row r="474" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="474" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A474" s="7"/>
       <c r="H474" s="3"/>
     </row>
-    <row r="475" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="475" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A475" s="7"/>
       <c r="H475" s="3"/>
     </row>
-    <row r="476" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A476" s="7"/>
       <c r="H476" s="3"/>
     </row>
-    <row r="477" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A477" s="7"/>
       <c r="H477" s="3"/>
     </row>
-    <row r="478" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A478" s="7"/>
       <c r="H478" s="3"/>
     </row>
-    <row r="479" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A479" s="7"/>
       <c r="H479" s="3"/>
     </row>
-    <row r="480" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A480" s="7"/>
       <c r="H480" s="3"/>
     </row>
-    <row r="481" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A481" s="7"/>
       <c r="H481" s="3"/>
     </row>
-    <row r="482" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="482" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A482" s="7"/>
       <c r="H482" s="3"/>
     </row>
-    <row r="483" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="483" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A483" s="7"/>
       <c r="H483" s="3"/>
     </row>
-    <row r="484" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="484" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A484" s="7"/>
       <c r="H484" s="3"/>
     </row>
-    <row r="485" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="485" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A485" s="7"/>
       <c r="H485" s="3"/>
     </row>
-    <row r="486" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="486" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A486" s="7"/>
       <c r="H486" s="3"/>
     </row>
-    <row r="487" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="487" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A487" s="7"/>
       <c r="H487" s="3"/>
     </row>
-    <row r="488" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="488" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A488" s="7"/>
       <c r="H488" s="3"/>
     </row>
-    <row r="489" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="489" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A489" s="7"/>
       <c r="H489" s="3"/>
     </row>
-    <row r="490" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="490" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A490" s="7"/>
       <c r="H490" s="3"/>
     </row>
-    <row r="491" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="491" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A491" s="7"/>
       <c r="H491" s="3"/>
     </row>
-    <row r="492" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="492" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A492" s="7"/>
       <c r="H492" s="3"/>
     </row>
-    <row r="493" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="493" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A493" s="7"/>
       <c r="H493" s="3"/>
     </row>
-    <row r="494" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="494" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A494" s="7"/>
       <c r="H494" s="3"/>
     </row>
-    <row r="495" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="495" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A495" s="7"/>
       <c r="H495" s="3"/>
     </row>
-    <row r="496" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="496" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A496" s="7"/>
       <c r="H496" s="3"/>
     </row>
-    <row r="497" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="497" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A497" s="7"/>
       <c r="H497" s="3"/>
     </row>
-    <row r="498" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="498" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A498" s="7"/>
       <c r="H498" s="3"/>
     </row>
-    <row r="499" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="499" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A499" s="7"/>
       <c r="H499" s="3"/>
     </row>
-    <row r="500" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="500" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A500" s="7"/>
       <c r="H500" s="3"/>
     </row>
-    <row r="501" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="501" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A501" s="7"/>
       <c r="H501" s="3"/>
     </row>
-    <row r="502" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="502" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A502" s="7"/>
       <c r="H502" s="3"/>
     </row>
-    <row r="503" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="503" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A503" s="7"/>
       <c r="H503" s="3"/>
     </row>
-    <row r="504" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="504" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A504" s="7"/>
       <c r="H504" s="3"/>
     </row>
-    <row r="505" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="505" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A505" s="7"/>
       <c r="H505" s="3"/>
     </row>
-    <row r="506" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="506" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A506" s="7"/>
       <c r="H506" s="3"/>
     </row>
-    <row r="507" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="507" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A507" s="7"/>
       <c r="H507" s="3"/>
     </row>
-    <row r="508" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="508" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A508" s="7"/>
       <c r="H508" s="3"/>
     </row>
-    <row r="509" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="509" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A509" s="7"/>
       <c r="H509" s="3"/>
     </row>
-    <row r="510" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="510" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A510" s="7"/>
       <c r="H510" s="3"/>
     </row>
-    <row r="511" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="511" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A511" s="7"/>
       <c r="H511" s="3"/>
     </row>
-    <row r="512" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="512" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A512" s="7"/>
       <c r="H512" s="3"/>
     </row>
-    <row r="513" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="513" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A513" s="7"/>
       <c r="H513" s="3"/>
     </row>
-    <row r="514" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="514" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A514" s="7"/>
       <c r="H514" s="3"/>
     </row>
-    <row r="515" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="515" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A515" s="7"/>
       <c r="H515" s="3"/>
     </row>
-    <row r="516" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="516" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A516" s="7"/>
       <c r="H516" s="3"/>
     </row>
-    <row r="517" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="517" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A517" s="7"/>
       <c r="H517" s="3"/>
     </row>
-    <row r="518" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="518" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A518" s="7"/>
       <c r="H518" s="3"/>
     </row>
-    <row r="519" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="519" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A519" s="7"/>
       <c r="H519" s="3"/>
     </row>
-    <row r="520" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="520" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A520" s="7"/>
       <c r="H520" s="3"/>
     </row>
-    <row r="521" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="521" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A521" s="7"/>
       <c r="H521" s="3"/>
     </row>
-    <row r="522" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="522" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A522" s="7"/>
       <c r="H522" s="3"/>
     </row>
-    <row r="523" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="523" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A523" s="7"/>
       <c r="H523" s="3"/>
     </row>
-    <row r="524" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="524" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A524" s="7"/>
       <c r="H524" s="3"/>
     </row>
-    <row r="525" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="525" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A525" s="7"/>
       <c r="H525" s="3"/>
     </row>
-    <row r="526" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="526" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A526" s="7"/>
       <c r="H526" s="3"/>
     </row>
-    <row r="527" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="527" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A527" s="7"/>
       <c r="H527" s="3"/>
     </row>
-    <row r="528" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="528" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A528" s="7"/>
       <c r="H528" s="3"/>
     </row>
-    <row r="529" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="529" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A529" s="7"/>
       <c r="H529" s="3"/>
     </row>
-    <row r="530" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="530" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A530" s="7"/>
       <c r="H530" s="3"/>
     </row>
-    <row r="531" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="531" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A531" s="7"/>
       <c r="H531" s="3"/>
     </row>
-    <row r="532" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="532" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A532" s="7"/>
       <c r="H532" s="3"/>
     </row>
-    <row r="533" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="533" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A533" s="7"/>
       <c r="H533" s="3"/>
     </row>
-    <row r="534" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="534" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A534" s="7"/>
       <c r="H534" s="3"/>
     </row>
-    <row r="535" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="535" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A535" s="7"/>
       <c r="H535" s="3"/>
     </row>
-    <row r="536" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="536" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A536" s="7"/>
       <c r="H536" s="3"/>
     </row>
-    <row r="537" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="537" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A537" s="7"/>
       <c r="H537" s="3"/>
     </row>
-    <row r="538" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="538" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A538" s="7"/>
       <c r="H538" s="3"/>
     </row>
-    <row r="539" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="539" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A539" s="7"/>
       <c r="H539" s="3"/>
     </row>
-    <row r="540" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="540" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A540" s="7"/>
       <c r="H540" s="3"/>
     </row>
-    <row r="541" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="541" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A541" s="7"/>
       <c r="H541" s="3"/>
     </row>
-    <row r="542" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="542" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A542" s="7"/>
       <c r="H542" s="3"/>
     </row>
-    <row r="543" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="543" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A543" s="7"/>
       <c r="H543" s="3"/>
     </row>
-    <row r="544" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="544" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A544" s="7"/>
       <c r="H544" s="3"/>
     </row>
-    <row r="545" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="545" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A545" s="7"/>
       <c r="H545" s="3"/>
     </row>
-    <row r="546" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="546" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A546" s="7"/>
       <c r="H546" s="3"/>
     </row>
-    <row r="547" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="547" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A547" s="7"/>
       <c r="H547" s="3"/>
     </row>
-    <row r="548" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="548" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A548" s="7"/>
       <c r="H548" s="3"/>
     </row>
-    <row r="549" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="549" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A549" s="7"/>
       <c r="H549" s="3"/>
     </row>
-    <row r="550" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="550" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A550" s="7"/>
       <c r="H550" s="3"/>
     </row>
-    <row r="551" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="551" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A551" s="7"/>
       <c r="H551" s="3"/>
     </row>
-    <row r="552" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="552" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A552" s="7"/>
       <c r="H552" s="3"/>
     </row>
-    <row r="553" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="553" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A553" s="7"/>
       <c r="H553" s="3"/>
     </row>
-    <row r="554" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="554" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A554" s="7"/>
       <c r="H554" s="3"/>
     </row>
-    <row r="555" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="555" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A555" s="7"/>
       <c r="H555" s="3"/>
     </row>
-    <row r="556" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="556" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A556" s="7"/>
       <c r="H556" s="3"/>
     </row>
-    <row r="557" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="557" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A557" s="7"/>
       <c r="H557" s="3"/>
     </row>
-    <row r="558" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="558" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A558" s="7"/>
       <c r="H558" s="3"/>
     </row>
-    <row r="559" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="559" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A559" s="7"/>
       <c r="H559" s="3"/>
     </row>
-    <row r="560" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="560" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A560" s="7"/>
       <c r="H560" s="3"/>
     </row>
-    <row r="561" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="561" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A561" s="7"/>
       <c r="H561" s="3"/>
     </row>
-    <row r="562" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="562" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A562" s="7"/>
       <c r="H562" s="3"/>
     </row>
-    <row r="563" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="563" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A563" s="7"/>
       <c r="H563" s="3"/>
     </row>
-    <row r="564" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="564" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A564" s="7"/>
       <c r="H564" s="3"/>
     </row>
-    <row r="565" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="565" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A565" s="7"/>
       <c r="H565" s="3"/>
     </row>
-    <row r="566" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="566" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A566" s="7"/>
       <c r="H566" s="3"/>
     </row>
-    <row r="567" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="567" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A567" s="7"/>
       <c r="H567" s="3"/>
     </row>
-    <row r="568" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="568" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A568" s="7"/>
       <c r="H568" s="3"/>
     </row>
-    <row r="569" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="569" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A569" s="7"/>
       <c r="H569" s="3"/>
     </row>
-    <row r="570" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="570" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A570" s="7"/>
       <c r="H570" s="3"/>
     </row>
-    <row r="571" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="571" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A571" s="7"/>
       <c r="H571" s="3"/>
     </row>
-    <row r="572" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="572" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A572" s="7"/>
       <c r="H572" s="3"/>
     </row>
-    <row r="573" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="573" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A573" s="7"/>
       <c r="H573" s="3"/>
     </row>
-    <row r="574" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="574" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A574" s="7"/>
       <c r="H574" s="3"/>
     </row>
-    <row r="575" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="575" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A575" s="7"/>
       <c r="H575" s="3"/>
     </row>
-    <row r="576" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="576" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A576" s="7"/>
       <c r="H576" s="3"/>
     </row>
-    <row r="577" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="577" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A577" s="7"/>
       <c r="H577" s="3"/>
     </row>
-    <row r="578" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="578" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A578" s="7"/>
       <c r="H578" s="3"/>
     </row>
-    <row r="579" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="579" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A579" s="7"/>
       <c r="H579" s="3"/>
     </row>
-    <row r="580" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="580" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A580" s="7"/>
       <c r="H580" s="3"/>
     </row>
-    <row r="581" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="581" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A581" s="7"/>
       <c r="H581" s="3"/>
     </row>
-    <row r="582" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="582" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A582" s="7"/>
       <c r="H582" s="3"/>
     </row>
-    <row r="583" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="583" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A583" s="7"/>
       <c r="H583" s="3"/>
     </row>
-    <row r="584" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="584" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A584" s="7"/>
       <c r="H584" s="3"/>
     </row>
-    <row r="585" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="585" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A585" s="7"/>
       <c r="H585" s="3"/>
     </row>
-    <row r="586" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="586" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A586" s="7"/>
       <c r="H586" s="3"/>
     </row>
-    <row r="587" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="587" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A587" s="7"/>
       <c r="H587" s="3"/>
     </row>
-    <row r="588" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="588" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A588" s="7"/>
       <c r="H588" s="3"/>
     </row>
-    <row r="589" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="589" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A589" s="7"/>
       <c r="H589" s="3"/>
     </row>
-    <row r="590" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="590" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A590" s="7"/>
       <c r="H590" s="3"/>
     </row>
-    <row r="591" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="591" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A591" s="7"/>
       <c r="H591" s="3"/>
     </row>
-    <row r="592" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="592" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A592" s="7"/>
       <c r="H592" s="3"/>
     </row>
-    <row r="593" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="593" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A593" s="7"/>
       <c r="H593" s="3"/>
     </row>
-    <row r="594" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="594" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A594" s="7"/>
       <c r="H594" s="3"/>
     </row>
-    <row r="595" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="595" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A595" s="7"/>
       <c r="H595" s="3"/>
     </row>
-    <row r="596" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="596" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A596" s="7"/>
       <c r="H596" s="3"/>
     </row>
-    <row r="597" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="597" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A597" s="7"/>
       <c r="H597" s="3"/>
     </row>
-    <row r="598" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="598" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A598" s="7"/>
       <c r="H598" s="3"/>
     </row>
-    <row r="599" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="599" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A599" s="7"/>
       <c r="H599" s="3"/>
     </row>
-    <row r="600" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="600" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A600" s="7"/>
       <c r="H600" s="3"/>
     </row>
-    <row r="601" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="601" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A601" s="7"/>
       <c r="H601" s="3"/>
     </row>
-    <row r="602" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="602" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A602" s="7"/>
       <c r="H602" s="3"/>
     </row>
-    <row r="603" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="603" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A603" s="7"/>
       <c r="H603" s="3"/>
     </row>
-    <row r="604" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="604" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A604" s="7"/>
       <c r="H604" s="3"/>
     </row>
-    <row r="605" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="605" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A605" s="7"/>
       <c r="H605" s="3"/>
     </row>
-    <row r="606" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="606" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A606" s="7"/>
       <c r="H606" s="3"/>
     </row>
-    <row r="607" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="607" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A607" s="7"/>
       <c r="H607" s="3"/>
     </row>
-    <row r="608" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="608" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A608" s="7"/>
       <c r="H608" s="3"/>
     </row>
-    <row r="609" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="609" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A609" s="7"/>
       <c r="H609" s="3"/>
     </row>
-    <row r="610" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="610" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A610" s="7"/>
       <c r="H610" s="3"/>
     </row>
-    <row r="611" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="611" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A611" s="7"/>
       <c r="H611" s="3"/>
     </row>
-    <row r="612" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="612" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A612" s="7"/>
       <c r="H612" s="3"/>
     </row>
-    <row r="613" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="613" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A613" s="7"/>
       <c r="H613" s="3"/>
     </row>
-    <row r="614" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="614" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A614" s="7"/>
       <c r="H614" s="3"/>
     </row>
-    <row r="615" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="615" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A615" s="7"/>
       <c r="H615" s="3"/>
     </row>
-    <row r="616" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="616" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A616" s="7"/>
       <c r="H616" s="3"/>
     </row>
-    <row r="617" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="617" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A617" s="7"/>
       <c r="H617" s="3"/>
     </row>
-    <row r="618" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="618" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A618" s="7"/>
       <c r="H618" s="3"/>
     </row>
-    <row r="619" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="619" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A619" s="7"/>
       <c r="H619" s="3"/>
     </row>
-    <row r="620" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="620" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A620" s="7"/>
       <c r="H620" s="3"/>
     </row>
-    <row r="621" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="621" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A621" s="7"/>
       <c r="H621" s="3"/>
     </row>
-    <row r="622" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="622" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A622" s="7"/>
       <c r="H622" s="3"/>
     </row>
-    <row r="623" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="623" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A623" s="7"/>
       <c r="H623" s="3"/>
     </row>
-    <row r="624" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="624" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A624" s="7"/>
       <c r="H624" s="3"/>
     </row>
-    <row r="625" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="625" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A625" s="7"/>
       <c r="H625" s="3"/>
     </row>
-    <row r="626" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="626" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A626" s="7"/>
       <c r="H626" s="3"/>
     </row>
-    <row r="627" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="627" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A627" s="7"/>
       <c r="H627" s="3"/>
     </row>
-    <row r="628" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="628" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A628" s="7"/>
       <c r="H628" s="3"/>
     </row>
-    <row r="629" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="629" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A629" s="7"/>
       <c r="H629" s="3"/>
     </row>
-    <row r="630" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="630" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A630" s="7"/>
       <c r="H630" s="3"/>
     </row>
-    <row r="631" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="631" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A631" s="7"/>
       <c r="H631" s="3"/>
     </row>
-    <row r="632" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="632" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A632" s="7"/>
       <c r="H632" s="3"/>
     </row>
-    <row r="633" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="633" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A633" s="7"/>
       <c r="H633" s="3"/>
     </row>
-    <row r="634" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="634" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A634" s="7"/>
       <c r="H634" s="3"/>
     </row>
-    <row r="635" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="635" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A635" s="7"/>
       <c r="H635" s="3"/>
     </row>
-    <row r="636" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="636" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A636" s="7"/>
       <c r="H636" s="3"/>
     </row>
-    <row r="637" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="637" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A637" s="7"/>
       <c r="H637" s="3"/>
     </row>
-    <row r="638" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="638" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A638" s="7"/>
       <c r="H638" s="3"/>
     </row>
-    <row r="639" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="639" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A639" s="7"/>
       <c r="H639" s="3"/>
     </row>
-    <row r="640" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="640" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A640" s="7"/>
       <c r="H640" s="3"/>
     </row>
-    <row r="641" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="641" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A641" s="7"/>
       <c r="H641" s="3"/>
     </row>
-    <row r="642" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="642" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A642" s="7"/>
       <c r="H642" s="3"/>
     </row>
-    <row r="643" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="643" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A643" s="7"/>
       <c r="H643" s="3"/>
     </row>
-    <row r="644" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="644" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A644" s="7"/>
       <c r="H644" s="3"/>
     </row>
-    <row r="645" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="645" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A645" s="7"/>
       <c r="H645" s="3"/>
     </row>
-    <row r="646" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="646" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A646" s="7"/>
       <c r="H646" s="3"/>
     </row>
-    <row r="647" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="647" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A647" s="7"/>
       <c r="H647" s="3"/>
     </row>
+    <row r="648" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A648" s="7">
+        <v>46318</v>
+      </c>
+    </row>
+    <row r="649" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A649" s="7"/>
+    </row>
+    <row r="650" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A650" s="7"/>
+    </row>
+    <row r="651" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A651" s="7"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I647" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Andrade Home Resort"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:I648" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.51181102362204722" right="0.51181102362204722" top="0.78740157480314965" bottom="0.78740157480314965" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <ignoredErrors>
@@ -7077,7 +7121,7 @@
   </ignoredErrors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{070D9A3B-D984-42A1-8AD7-CE92EBF09B76}">
           <x14:formula1>
             <xm:f>Corretores!$A$2:$A$25</xm:f>

</xml_diff>